<commit_message>
dev ++ ----------- + connect enhance 7
</commit_message>
<xml_diff>
--- a/utility_core/static/src/Migration_Template.xlsx
+++ b/utility_core/static/src/Migration_Template.xlsx
@@ -649,7 +649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1004"/>
+  <dimension ref="A1:W1004"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -713,6 +713,16 @@
       <c r="R3" s="7" t="inlineStr">
         <is>
           <t>بيانات اضافية</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>بيانات اضافية</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>بيانات القراءة</t>
         </is>
       </c>
     </row>
@@ -817,6 +827,21 @@
           <t>مرجع المالك القديم</t>
         </is>
       </c>
+      <c r="U4" s="32" t="inlineStr">
+        <is>
+          <t>رمز المحول المرتبط</t>
+        </is>
+      </c>
+      <c r="V4" s="32" t="inlineStr">
+        <is>
+          <t>القراءة الحالية</t>
+        </is>
+      </c>
+      <c r="W4" s="32" t="inlineStr">
+        <is>
+          <t>تاريخ آخر قراءة</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="26" t="n"/>
@@ -834,6 +859,9 @@
       <c r="O5" s="27" t="n"/>
       <c r="Q5" s="27" t="n"/>
       <c r="T5" s="26" t="n"/>
+      <c r="U5" s="26" t="n"/>
+      <c r="V5" s="26" t="n"/>
+      <c r="W5" s="26" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="B6" s="26" t="n"/>
@@ -851,6 +879,9 @@
       <c r="O6" s="27" t="n"/>
       <c r="Q6" s="27" t="n"/>
       <c r="T6" s="26" t="n"/>
+      <c r="U6" s="26" t="n"/>
+      <c r="V6" s="26" t="n"/>
+      <c r="W6" s="26" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="B7" s="26" t="n"/>
@@ -868,6 +899,9 @@
       <c r="O7" s="27" t="n"/>
       <c r="Q7" s="27" t="n"/>
       <c r="T7" s="26" t="n"/>
+      <c r="U7" s="26" t="n"/>
+      <c r="V7" s="26" t="n"/>
+      <c r="W7" s="26" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="B8" s="26" t="n"/>
@@ -885,6 +919,9 @@
       <c r="O8" s="27" t="n"/>
       <c r="Q8" s="27" t="n"/>
       <c r="T8" s="26" t="n"/>
+      <c r="U8" s="26" t="n"/>
+      <c r="V8" s="26" t="n"/>
+      <c r="W8" s="26" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="B9" s="26" t="n"/>
@@ -17820,13 +17857,14 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:T4"/>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="A1:S1"/>
     <mergeCell ref="R3:S3"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="M3:Q3"/>
     <mergeCell ref="A2:S2"/>
+    <mergeCell ref="V3:W3"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="G5:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -17849,7 +17887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -17860,7 +17898,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="28" t="inlineStr">
         <is>
-          <t>تعليمات استيراد المشتركين — عقد v4</t>
+          <t>تعليمات استيراد المشتركين — عقد v6</t>
         </is>
       </c>
       <c r="B1" s="29" t="inlineStr"/>
@@ -17884,7 +17922,7 @@
         </is>
       </c>
       <c r="B3" s="29" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -17947,9 +17985,42 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1"/>
-    <row r="10" ht="22" customHeight="1"/>
-    <row r="11" ht="22" customHeight="1"/>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>رمز المحول المرتبط</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>اختياري. يجب أن يكون المحول مرفوعاً مسبقاً في شاشة تهيئة المحولات؛ يُربط العميل بالمسار التابع للمحول (يُنشأ المسار الافتراضي تلقائياً عند عدم وجوده).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>القراءة الحالية</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>اختياري. القراءة الحالية للعداد؛ تُسجَّل على العداد وعلى الحساب بعد التوريد. الفراغ لا يغيّر شيئاً والصفر قراءة صحيحة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>تاريخ آخر قراءة</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>اختياري. تاريخ آخر قراءة مسجلة بصيغة YYYY-MM-DD؛ يُسجَّل على العداد وعلى الحساب (آخر تاريخ قراءة).</t>
+        </is>
+      </c>
+    </row>
     <row r="12" ht="22" customHeight="1"/>
     <row r="13" ht="24" customHeight="1"/>
     <row r="14" ht="18" customHeight="1"/>

</xml_diff>